<commit_message>
chore: ajusta Modelo.xlsx (estilos e Tabela1)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modelo.xlsx
+++ b/Modelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/es/Documents/conta_de_gastos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{190D76D9-EE04-2D44-AD00-FFA73E90EB62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4494AE0-67CC-1E48-AFAE-50B3C9F6D172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="1740" windowWidth="29000" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="100" yWindow="1060" windowWidth="29000" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Extrato" sheetId="1" r:id="rId1"/>
@@ -612,7 +612,18 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Título" xfId="2" builtinId="15"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -858,16 +869,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6F26D33F-9FC5-4442-A295-DA7C474F689D}" name="Tabela1" displayName="Tabela1" ref="A7:G503" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6F26D33F-9FC5-4442-A295-DA7C474F689D}" name="Tabela1" displayName="Tabela1" ref="A7:G503" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A7:G503" xr:uid="{6F26D33F-9FC5-4442-A295-DA7C474F689D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{2E98334D-5CFA-F24B-AE4B-A17AACBC104A}" name="Fonte" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{985FDF7A-260E-054A-972E-05483EC5CD50}" name="Data" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{C0EB3965-5FCC-834F-B8DB-8D424B2F1818}" name="Transcrição" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{6E1105DD-6855-8843-9B76-D7978BF1910D}" name="Iniciais" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{E257224B-B774-074E-B6D4-DE58D555A465}" name="Natureza" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{E28D192D-BA01-AD4D-BC50-ABCAC1F70F3F}" name="Descrição" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{E56D9CAE-DF36-E140-B4E6-73A60CB0B633}" name="Valor" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{2E98334D-5CFA-F24B-AE4B-A17AACBC104A}" name="Fonte" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{985FDF7A-260E-054A-972E-05483EC5CD50}" name="Data" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{C0EB3965-5FCC-834F-B8DB-8D424B2F1818}" name="Transcrição" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{6E1105DD-6855-8843-9B76-D7978BF1910D}" name="Iniciais" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{E257224B-B774-074E-B6D4-DE58D555A465}" name="Natureza" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{E28D192D-BA01-AD4D-BC50-ABCAC1F70F3F}" name="Descrição" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{E56D9CAE-DF36-E140-B4E6-73A60CB0B633}" name="Valor" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -24215,8 +24226,8 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="1" id="{BD7AF845-0326-764F-9056-91F2F7A89C19}">
-            <xm:f>OR(AND($E31&lt;&gt;"",ISNA(MATCH($E31,Naturezas!$B$3:$B$32,0))),AND($E31="",COUNTA($A31:$C31,$F31:$G31)&gt;0))</xm:f>
+          <x14:cfRule type="expression" priority="1" id="{9CA8196D-BD2B-BC45-BDD8-5D56FC47C910}">
+            <xm:f>OR(AND($E8&lt;&gt;"",ISNA(MATCH($E8,Naturezas!$B$3:$B$32,0))),AND($E8="",COUNTA($A8:$D8,$F8:$G8)&gt;0))</xm:f>
             <x14:dxf>
               <font>
                 <color rgb="FF9C0006"/>
@@ -24229,7 +24240,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E31:E503</xm:sqref>
+          <xm:sqref>E8:E503</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
feat(modelo): Modelo com totais na linha dos títulos da Tabela1 + writer robusto a re-saves
Modelo.xlsx atualizado manualmente (item 18): fórmulas de totais movidas
para a linha dos títulos (J8/M8) para sobreviverem a filtros da Tabela1;
re-salvo com a aba Extrato ativa. public/Modelo.xlsx e a fixture de testes
sincronizados com o mesmo hash (sem drift). Contrato de injeção validado:
Tabela1 A8:H504, B2 s=40, B3 s=45, calcPr presente, A:H sem fórmulas no
corpo.

O re-save expôs duas fragilidades do writer, corrigidas: a injeção de B3
casava um literal exato com shared string (o re-save esvaziou a célula) e
agora usa regex que aceita ambas as formas; forcarAbaExtratoAtiva insere
activeTab="0" quando o atributo não existe no workbookView.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QPCiJawDbLQ7aX1zPopds
</commit_message>
<xml_diff>
--- a/Modelo.xlsx
+++ b/Modelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/es/Documents/conta_de_gastos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3690F970-A296-6840-8BCF-20DDBC7100C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39083A0D-9768-E445-8EE1-CEEA4E189564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="-19780" windowWidth="29000" windowHeight="18060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="80" yWindow="1060" windowWidth="29000" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Extrato" sheetId="1" r:id="rId1"/>
@@ -35,10 +35,9 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="2">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
@@ -49,30 +48,16 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="1">
-    <bk>
-      <rc t="2" v="0"/>
-    </bk>
-  </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="109">
   <si>
     <t>Saldo inicial</t>
   </si>
@@ -317,9 +302,6 @@
     <t>Dados de apoio</t>
   </si>
   <si>
-    <t>Somatória</t>
-  </si>
-  <si>
     <t>Lançamentos</t>
   </si>
   <si>
@@ -341,9 +323,6 @@
     <t>Referência</t>
   </si>
   <si>
-    <t>2026-06</t>
-  </si>
-  <si>
     <t>Ref.</t>
   </si>
   <si>
@@ -357,6 +336,54 @@
   </si>
   <si>
     <t>Suporte 4</t>
+  </si>
+  <si>
+    <t>Descrição curta</t>
+  </si>
+  <si>
+    <t>Gastos com consultas, exames, remédios, tratamentos, plano de saúde etc.</t>
+  </si>
+  <si>
+    <t>Gastos com roupas, sapatos, indumentária em geral</t>
+  </si>
+  <si>
+    <t>Gastos ordinários (assinaturas, transporte, refeições, etc.)</t>
+  </si>
+  <si>
+    <t>Receitas e despesas vinculadas ao trabalho profissional e previdência privada</t>
+  </si>
+  <si>
+    <t>Gastos com cursos anuais, convívios, retiros, viagens, despesas extraordinárias etc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastos com combustível, pedágio, limpeza, manutenção, etc. </t>
+  </si>
+  <si>
+    <t>Pagamento de ordenados</t>
+  </si>
+  <si>
+    <t>Pagamento de despesas com comestiveis para a casa em geral</t>
+  </si>
+  <si>
+    <t>Conta de energia</t>
+  </si>
+  <si>
+    <t>Conta de água</t>
+  </si>
+  <si>
+    <t>Conta de gás</t>
+  </si>
+  <si>
+    <t>Conta de internet e telefonia</t>
+  </si>
+  <si>
+    <t>Custos com manutenção</t>
+  </si>
+  <si>
+    <t>Custos para consertos e melhorias em geral nas instalações da casa</t>
+  </si>
+  <si>
+    <t>Custos com jardinagem, faxina, materiais de limpeza, peças e insumos para manutenção etc.</t>
   </si>
 </sst>
 </file>
@@ -845,64 +872,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <rv s="0">
-    <v>13</v>
-    <v>3</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_error">
-    <k n="errorType" t="i"/>
-    <k n="subType" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6F26D33F-9FC5-4442-A295-DA7C474F689D}" name="Tabela1" displayName="Tabela1" ref="A8:H504" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A8:H504" xr:uid="{6F26D33F-9FC5-4442-A295-DA7C474F689D}"/>
@@ -1178,23 +1147,21 @@
   <sheetData>
     <row r="1" spans="1:36" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="30" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B2" s="40"/>
       <c r="O2"/>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="B3" s="45" t="s">
-        <v>89</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="B3" s="45"/>
       <c r="O3"/>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.2">
@@ -1224,24 +1191,24 @@
     </row>
     <row r="7" spans="1:36" ht="24" x14ac:dyDescent="0.3">
       <c r="A7" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H7" s="2"/>
       <c r="J7" s="30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
       <c r="Q7" s="30" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="X7" s="3"/>
       <c r="AA7" s="30" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="AC7" s="3"/>
     </row>
@@ -1256,10 +1223,10 @@
         <v>6</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>4</v>
@@ -1270,28 +1237,30 @@
       <c r="H8" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="J8" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="K8" s="28" t="s">
-        <v>81</v>
+      <c r="J8" s="27" t="str" cm="1">
+        <f t="array" ref="J8:K8">_xlfn.LET(_xlpm.nat,Tabela1[Natureza],_xlpm.hdr,_xlfn.HSTACK("Natureza","Somatória"),IF(SUM(--(_xlpm.nat&lt;&gt;""))=0,_xlpm.hdr,_xlfn.LET(_xlpm.u,_xlfn.UNIQUE(_xlfn._xlws.FILTER(_xlpm.nat,_xlpm.nat&lt;&gt;"")),_xlpm.k,IF(_xlpm.u="RR",0,_xlfn.XMATCH(_xlpm.u,_xlpm.u)),_xlpm.n,_xlfn.SORTBY(_xlpm.u,_xlpm.k,1),_xlpm.s,SUMIF(Tabela1[Natureza],_xlpm.n,Tabela1[Valor]),_xlfn.VSTACK(_xlpm.hdr,_xlfn.HSTACK(_xlpm.n,_xlpm.s),_xlfn.HSTACK("TOTAL &gt;&gt;&gt;",SUM(_xlpm.s))))))</f>
+        <v>Natureza</v>
+      </c>
+      <c r="K8" s="28" t="str">
+        <v>Somatória</v>
       </c>
       <c r="L8" s="18"/>
-      <c r="M8" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="N8" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="O8" s="27" t="s">
-        <v>7</v>
+      <c r="M8" s="27" t="str" cm="1">
+        <f t="array" ref="M8:O8">_xlfn.LET(_xlpm.natcol,Tabela1[Natureza],_xlpm.hdr,_xlfn.HSTACK("Natureza","Descrição","Valor"),IF(SUM(--(_xlpm.natcol&lt;&gt;""))=0,_xlpm.hdr,_xlfn.LET(_xlpm.d,_xlfn._xlws.FILTER(_xlfn.HSTACK(Tabela1[Natureza],Tabela1[Descrição],Tabela1[Valor]),_xlpm.natcol&lt;&gt;""),_xlpm.ordem,_xlfn.XMATCH(_xlfn.CHOOSECOLS(_xlpm.d,1),_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(J8),1)),_xlpm.sorted,_xlfn.SORTBY(_xlpm.d,_xlpm.ordem,1,ABS(_xlfn.CHOOSECOLS(_xlpm.d,3)),-1),_xlpm.nat,_xlfn.CHOOSECOLS(_xlpm.sorted,1),_xlpm.r,ROWS(_xlpm.sorted),_xlpm.body,_xlfn.DROP(_xlfn.REDUCE(_xlfn.HSTACK("","",""),_xlfn.SEQUENCE(_xlpm.r),_xlfn.LAMBDA(_xlpm.acc,_xlpm.i,IF(AND(_xlpm.i&gt;1,INDEX(_xlpm.nat,_xlpm.i)&lt;&gt;INDEX(_xlpm.nat,_xlpm.i-1)),_xlfn.VSTACK(_xlpm.acc,_xlfn.HSTACK("","",""),INDEX(_xlpm.sorted,_xlpm.i,0)),_xlfn.VSTACK(_xlpm.acc,INDEX(_xlpm.sorted,_xlpm.i,0))))),1),_xlfn.VSTACK(_xlpm.hdr,_xlpm.body))))</f>
+        <v>Natureza</v>
+      </c>
+      <c r="N8" s="27" t="str">
+        <v>Descrição</v>
+      </c>
+      <c r="O8" s="27" t="str">
+        <v>Valor</v>
       </c>
       <c r="P8" s="19"/>
       <c r="Q8" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="R8" s="22" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="S8" s="22" t="s">
         <v>8</v>
@@ -1314,10 +1283,10 @@
       </c>
       <c r="Z8"/>
       <c r="AA8" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AB8" s="22" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="AC8" s="22" t="s">
         <v>12</v>
@@ -1339,15 +1308,9 @@
       <c r="F9" s="11"/>
       <c r="G9" s="11"/>
       <c r="H9" s="43"/>
-      <c r="J9" s="31" t="e" cm="1" vm="1">
-        <f t="array" ref="J9">_xlfn.LET(_xlpm.u,_xlfn.UNIQUE(_xlfn._xlws.FILTER(Tabela1[Natureza],Tabela1[Natureza]&lt;&gt;"")),_xlpm.k,IF(_xlpm.u="RR",0,_xlfn.XMATCH(_xlpm.u,_xlpm.u)),_xlpm.n,_xlfn.SORTBY(_xlpm.u,_xlpm.k,1),_xlpm.s,SUMIF(Tabela1[Natureza],_xlpm.n,Tabela1[Valor]),_xlfn.VSTACK(_xlfn.HSTACK(_xlpm.n,_xlpm.s),_xlfn.HSTACK("TOTAL &gt;&gt;&gt;",SUM(_xlpm.s))))</f>
-        <v>#VALUE!</v>
-      </c>
+      <c r="J9" s="31"/>
       <c r="K9" s="34"/>
-      <c r="M9" s="31" t="e" cm="1" vm="1">
-        <f t="array" ref="M9">_xlfn.LET(_xlpm.d,_xlfn._xlws.FILTER(_xlfn.HSTACK(Tabela1[Natureza],Tabela1[Descrição],Tabela1[Valor]),Tabela1[Natureza]&lt;&gt;""),_xlpm.ordem,_xlfn.XMATCH(_xlfn.CHOOSECOLS(_xlpm.d,1),_xlfn.CHOOSECOLS(_xlfn.ANCHORARRAY(J9),1)),_xlpm.sorted,_xlfn.SORTBY(_xlpm.d,_xlpm.ordem,1,ABS(_xlfn.CHOOSECOLS(_xlpm.d,3)),-1),_xlpm.nat,_xlfn.CHOOSECOLS(_xlpm.sorted,1),_xlpm.r,ROWS(_xlpm.sorted),_xlfn.DROP(_xlfn.REDUCE(_xlfn.HSTACK("","",""),_xlfn.SEQUENCE(_xlpm.r),_xlfn.LAMBDA(_xlpm.acc,_xlpm.i,IF(AND(_xlpm.i&gt;1,INDEX(_xlpm.nat,_xlpm.i)&lt;&gt;INDEX(_xlpm.nat,_xlpm.i-1)),_xlfn.VSTACK(_xlpm.acc,_xlfn.HSTACK("","",""),INDEX(_xlpm.sorted,_xlpm.i,0)),_xlfn.VSTACK(_xlpm.acc,INDEX(_xlpm.sorted,_xlpm.i,0))))),1))</f>
-        <v>#VALUE!</v>
-      </c>
+      <c r="M9" s="31"/>
       <c r="N9" s="31"/>
       <c r="O9" s="33"/>
       <c r="P9" s="3"/>
@@ -39551,25 +39514,26 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F054F059-67C5-3A41-B464-25C60F37A0F2}">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" customWidth="1"/>
     <col min="3" max="3" width="7.5" customWidth="1"/>
     <col min="4" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="70.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
@@ -39585,8 +39549,11 @@
       <c r="E2" s="21" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F2" s="21" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
         <v>14</v>
       </c>
@@ -39602,8 +39569,11 @@
       <c r="E3" s="20" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F3" s="20" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>19</v>
       </c>
@@ -39619,8 +39589,9 @@
       <c r="E4" s="7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F4" s="7"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>21</v>
       </c>
@@ -39636,8 +39607,9 @@
       <c r="E5" s="7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>23</v>
       </c>
@@ -39653,8 +39625,9 @@
       <c r="E6" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6" s="8"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>27</v>
       </c>
@@ -39670,8 +39643,11 @@
       <c r="E7" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F7" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>29</v>
       </c>
@@ -39687,8 +39663,11 @@
       <c r="E8" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8" s="8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>31</v>
       </c>
@@ -39704,8 +39683,11 @@
       <c r="E9" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F9" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
         <v>33</v>
       </c>
@@ -39721,8 +39703,11 @@
       <c r="E10" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
         <v>35</v>
       </c>
@@ -39738,8 +39723,9 @@
       <c r="E11" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F11" s="8"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
         <v>37</v>
       </c>
@@ -39755,8 +39741,11 @@
       <c r="E12" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F12" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>39</v>
       </c>
@@ -39772,8 +39761,9 @@
       <c r="E13" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
         <v>41</v>
       </c>
@@ -39789,8 +39779,9 @@
       <c r="E14" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14" s="8"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>43</v>
       </c>
@@ -39806,8 +39797,9 @@
       <c r="E15" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
         <v>45</v>
       </c>
@@ -39823,8 +39815,9 @@
       <c r="E16" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F16" s="8"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>47</v>
       </c>
@@ -39840,8 +39833,9 @@
       <c r="E17" s="7" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17" s="7"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>50</v>
       </c>
@@ -39857,8 +39851,9 @@
       <c r="E18" s="7" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
         <v>52</v>
       </c>
@@ -39874,8 +39869,9 @@
       <c r="E19" s="7" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
         <v>54</v>
       </c>
@@ -39891,8 +39887,9 @@
       <c r="E20" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F20" s="8"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
         <v>56</v>
       </c>
@@ -39908,8 +39905,11 @@
       <c r="E21" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F21" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
         <v>58</v>
       </c>
@@ -39925,8 +39925,11 @@
       <c r="E22" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F22" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>60</v>
       </c>
@@ -39942,8 +39945,9 @@
       <c r="E23" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
         <v>62</v>
       </c>
@@ -39959,8 +39963,11 @@
       <c r="E24" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F24" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
         <v>64</v>
       </c>
@@ -39976,8 +39983,11 @@
       <c r="E25" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F25" s="8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
         <v>66</v>
       </c>
@@ -39993,8 +40003,11 @@
       <c r="E26" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F26" s="8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
         <v>68</v>
       </c>
@@ -40010,8 +40023,11 @@
       <c r="E27" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F27" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
         <v>70</v>
       </c>
@@ -40027,8 +40043,11 @@
       <c r="E28" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F28" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="8" t="s">
         <v>72</v>
       </c>
@@ -40044,8 +40063,11 @@
       <c r="E29" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F29" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
         <v>41</v>
       </c>
@@ -40061,8 +40083,9 @@
       <c r="E30" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F30" s="8"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>74</v>
       </c>
@@ -40078,8 +40101,9 @@
       <c r="E31" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F31" s="8"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
         <v>76</v>
       </c>
@@ -40094,6 +40118,9 @@
       </c>
       <c r="E32" s="8" t="s">
         <v>49</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(colinha): descrição "DL" do Modelo.xlsx aparece na colinha de Naturezas
O usuário adicionou a descrição da natureza "DL" na aba Naturezas do
Modelo.xlsx (raiz), mas a colinha lê de public/Modelo.xlsx — que estava
defasado (drift raiz↔public, mesmo padrão do fix c455539). Copia o
Modelo.xlsx da raiz para public/ (agora idênticos) e atualiza o teste de
integração TL-T5-1 de 15 para 16 entradas com descrição não-vazia.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modelo.xlsx
+++ b/Modelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/es/Documents/conta_de_gastos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39083A0D-9768-E445-8EE1-CEEA4E189564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4DA68B-377F-8B47-9323-21A7055495E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="1060" windowWidth="29000" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="80" yWindow="1060" windowWidth="29000" windowHeight="18060" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Extrato" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="110">
   <si>
     <t>Saldo inicial</t>
   </si>
@@ -384,6 +384,9 @@
   </si>
   <si>
     <t>Custos com jardinagem, faxina, materiais de limpeza, peças e insumos para manutenção etc.</t>
+  </si>
+  <si>
+    <t>Subvenções e doações para iniciativas apostólicas, ajudas familiares etc.</t>
   </si>
 </sst>
 </file>
@@ -39815,7 +39818,9 @@
       <c r="E16" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="8"/>
+      <c r="F16" s="8" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">

</xml_diff>

<commit_message>
fix(modelo): re-salva Modelo desagrupado e sincroniza public/ + fixture
O .xlsx exportado abria com abas AGRUPADAS (sheet1 + sheet3 selecionadas)
e nesse modo o Excel bloqueia editar/excluir linhas da tabela. O
public/Modelo.xlsx estava salvo com tabSelected="1" na sheet3; o writer
força a seleção na sheet1 mas não limpava a sheet3, então o gerado saía
com duas abas selecionadas = agrupado.

Modelo.xlsx re-salvo com só a aba Extrato ativa. public/Modelo.xlsx (usado
no export) e a fixture de testes sincronizados ao mesmo hash — estavam os
três com hashes distintos (drift). Export regenerado: só sheet1 selecionada.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modelo.xlsx
+++ b/Modelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/es/Documents/conta_de_gastos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4DA68B-377F-8B47-9323-21A7055495E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1817F3E6-62F9-9F4A-9951-EB39E14C2F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="1060" windowWidth="29000" windowHeight="18060" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="80" yWindow="1060" windowWidth="29000" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Extrato" sheetId="1" r:id="rId1"/>

</xml_diff>